<commit_message>
Removed bar height column from template_survey_bargraph.xlsx; updated BarGraph* code accordingly
</commit_message>
<xml_diff>
--- a/src/main/resources/template_survey_bargraph.xlsx
+++ b/src/main/resources/template_survey_bargraph.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomma\saige\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898A7D3D-83FA-487C-A823-7BBC4C4C0FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A82DA39D-3833-4E5E-87B2-9FDEF32395AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EF544F7F-FE12-4575-9343-7880C024C4F5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>percentage_1</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>percentage_3</t>
-  </si>
-  <si>
-    <t>bar height (60 by default)</t>
   </si>
   <si>
     <t>imagename</t>
@@ -283,7 +280,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -293,6 +290,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -610,350 +610,326 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3580F207-1E93-4B18-BC79-037CEC09EC36}">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" customWidth="1"/>
     <col min="2" max="2" width="23.77734375" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="13.109375" customWidth="1"/>
-    <col min="6" max="6" width="15.21875" customWidth="1"/>
-    <col min="7" max="7" width="35.5546875" customWidth="1"/>
-    <col min="8" max="8" width="39.33203125" customWidth="1"/>
-    <col min="9" max="10" width="22.44140625" customWidth="1"/>
-    <col min="11" max="11" width="23.21875" customWidth="1"/>
-    <col min="12" max="12" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" customWidth="1"/>
+    <col min="6" max="6" width="35.5546875" customWidth="1"/>
+    <col min="7" max="7" width="39.33203125" customWidth="1"/>
+    <col min="8" max="9" width="22.44140625" customWidth="1"/>
+    <col min="10" max="10" width="23.21875" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="1"/>
+      <c r="C2">
+        <v>0</v>
+      </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>60</v>
-      </c>
-      <c r="F2">
-        <v>4</v>
-      </c>
-      <c r="G2" s="1">
-        <v>36</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="F2" s="1">
+        <v>84</v>
+      </c>
+      <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="1"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J2" s="2"/>
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>960</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>12</v>
+      </c>
+      <c r="F3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>576</v>
       </c>
-      <c r="D3">
-        <v>12</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>36</v>
-      </c>
-      <c r="G3">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>960</v>
+      <c r="C4">
+        <v>4</v>
       </c>
       <c r="D4">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="E4">
         <v>40</v>
       </c>
       <c r="F4">
-        <v>7</v>
-      </c>
-      <c r="G4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>11</v>
       </c>
       <c r="B5">
         <v>960</v>
       </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
       <c r="D5">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="F5">
-        <v>27</v>
-      </c>
-      <c r="G5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>960</v>
       </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
       <c r="D6">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E6">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>960</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>32</v>
+      </c>
+      <c r="F7">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>13</v>
-      </c>
-      <c r="B7">
-        <v>576</v>
-      </c>
-      <c r="D7">
-        <v>12</v>
-      </c>
-      <c r="E7">
-        <v>30</v>
-      </c>
-      <c r="F7">
-        <v>36</v>
-      </c>
-      <c r="G7">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>14</v>
       </c>
       <c r="B8">
         <v>960</v>
       </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
       <c r="D8">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="F8">
-        <v>17</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9">
         <v>960</v>
       </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
       <c r="D9">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="E9">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F9">
-        <v>7</v>
-      </c>
-      <c r="G9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <v>960</v>
       </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
       <c r="D10">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="E10">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="F10">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1">
+        <v>960</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>28</v>
+      </c>
+      <c r="F11" s="1">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="G10">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>50</v>
-      </c>
-      <c r="F11">
-        <v>14</v>
-      </c>
-      <c r="G11" s="1">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>18</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G29" s="3"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F28" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A13:G22"/>
+    <mergeCell ref="A13:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>